<commit_message>
feat: Update the delete
</commit_message>
<xml_diff>
--- a/growie_app/public/file/Sample Stocks Template with Data.xlsx
+++ b/growie_app/public/file/Sample Stocks Template with Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/32da6388213ebdb1/Growe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{B00D6C87-FDB2-491E-8F4F-0549F9C0EDBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C2ACD35-B578-4044-A258-80C31DD560B7}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{B00D6C87-FDB2-491E-8F4F-0549F9C0EDBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5BE8980-1A22-48DC-AF43-B4134526FD0D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Shares Breakdown (Scope Markets" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shares Breakdown (Scope Markets'!$A$2:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shares Breakdown (Scope Markets'!$A$2:$H$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="26">
   <si>
     <t>Purchase Dates</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Current Price</t>
   </si>
   <si>
-    <t>Initial Investment Value</t>
-  </si>
-  <si>
     <t>Goal</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
   </si>
   <si>
     <t>KES</t>
-  </si>
-  <si>
-    <t>Change in Investment Value</t>
   </si>
   <si>
     <t>Purchased Stocks</t>
@@ -126,14 +120,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="d&quot;-&quot;mmm&quot;-&quot;yy"/>
     <numFmt numFmtId="165" formatCode="[$$]#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$Ksh]#,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -144,6 +137,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -151,6 +145,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -158,18 +153,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Trebuchet MS"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -284,10 +274,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -311,32 +300,29 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -553,7 +539,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I965"/>
+  <dimension ref="A1:H965"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.140625" customWidth="1"/>
@@ -561,24 +547,22 @@
     <col min="3" max="4" width="12.5703125" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" customWidth="1"/>
-    <col min="10" max="10" width="3.85546875" customWidth="1"/>
+    <col min="9" max="9" width="3.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+    <row r="1" spans="1:8" s="13" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A1" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
       <c r="H1" s="16"/>
-      <c r="I1" s="17"/>
     </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -598,338 +582,290 @@
         <v>5</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>8</v>
-      </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>45959</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
       </c>
       <c r="E3" s="11">
         <v>5</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="17">
         <v>95.76</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="12">
-        <f>E3*F3</f>
-        <v>478.8</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>11</v>
+        <v>22</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>45959</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" s="11">
         <v>10</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="17">
         <v>208.42</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="12">
-        <f t="shared" ref="H4:H11" si="0">E4*F4</f>
-        <v>2084.1999999999998</v>
-      </c>
-      <c r="I4" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>45959</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" s="11">
         <v>10</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="17">
         <v>461.51</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="12">
-        <f t="shared" si="0"/>
-        <v>4615.1000000000004</v>
-      </c>
-      <c r="I5" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>45959</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E6" s="11">
         <v>10</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="17">
         <v>269.7</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="12">
-        <f t="shared" si="0"/>
-        <v>2697</v>
-      </c>
-      <c r="I6" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>45959</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" s="11">
         <v>1</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="17">
         <v>3920</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="12">
-        <f t="shared" si="0"/>
-        <v>3920</v>
-      </c>
-      <c r="I7" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>45992</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>10</v>
       </c>
       <c r="E8" s="11">
         <v>5</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="17">
         <v>86.57</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="12">
-        <f t="shared" si="0"/>
-        <v>432.84999999999997</v>
-      </c>
-      <c r="I8" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>45954</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="11">
         <v>10000</v>
       </c>
-      <c r="F9" s="12">
-        <v>0.216</v>
+      <c r="F9" s="17">
+        <v>28.1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="12">
-        <f t="shared" si="0"/>
-        <v>2160</v>
-      </c>
-      <c r="I9" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>45959</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E10" s="11">
         <v>500</v>
       </c>
-      <c r="F10" s="12">
-        <v>2.92</v>
+      <c r="F10" s="17">
+        <v>370</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" s="12">
-        <f t="shared" si="0"/>
-        <v>1460</v>
-      </c>
-      <c r="I10" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>45992</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" s="11">
         <v>3000</v>
       </c>
-      <c r="F11" s="12">
-        <v>0.21</v>
+      <c r="F11" s="17">
+        <v>27.5</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" s="12">
-        <f t="shared" si="0"/>
-        <v>630</v>
-      </c>
-      <c r="I11" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>45959</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="11">
         <v>6000</v>
       </c>
-      <c r="F12" s="12">
-        <v>0.39</v>
+      <c r="F12" s="18">
+        <v>51</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="12">
-        <f>E12*F12</f>
-        <v>2340</v>
-      </c>
-      <c r="I12" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
-      <c r="E13" s="14">
+      <c r="E13" s="12">
         <f>SUM(E3:E12)</f>
         <v>19541</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="13">
-        <f>SUM(H3:H12)</f>
-        <v>20817.95</v>
-      </c>
-      <c r="I13" s="3"/>
+      <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="16" spans="1:9" s="18" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A16" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:8" s="13" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A16" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
       <c r="H16" s="16"/>
-      <c r="I16" s="17"/>
     </row>
-    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>3</v>
@@ -944,13 +880,10 @@
         <v>6</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>45992</v>
       </c>
@@ -958,24 +891,25 @@
         <v>46083</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E18" s="5">
         <v>1500</v>
       </c>
-      <c r="F18" s="6">
-        <v>0.21</v>
-      </c>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="3" t="s">
-        <v>11</v>
+      <c r="F18" s="17">
+        <v>25.5</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="4"/>
@@ -983,10 +917,9 @@
       <c r="E19" s="5"/>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="3"/>
+      <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="4"/>
@@ -994,21 +927,20 @@
       <c r="E20" s="5"/>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="3"/>
+      <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1943,14 +1875,14 @@
     <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A2:I3" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I3">
+  <autoFilter ref="A2:H3" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H3">
       <sortCondition ref="A2:A3"/>
     </sortState>
   </autoFilter>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A3:A12 A18:B18" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>